<commit_message>
Disable fill tables and ignore sync logs
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Par-SYS_CO2price.xlsx
+++ b/SuppXLS/Scen_Par-SYS_CO2price.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A379DED-1777-44D2-9C57-3539F3A8AF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7FECC3-EB8C-4A13-8278-987EFC96EF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="25760" windowHeight="15440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="24" r:id="rId1"/>
@@ -433,7 +433,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -721,6 +721,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -730,7 +731,6 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1854,12 +1854,12 @@
       <c r="Z15" s="12"/>
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
       <c r="G16" s="14"/>
@@ -1943,11 +1943,11 @@
       <c r="A19" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
       <c r="E19" s="19"/>
       <c r="F19" s="19"/>
       <c r="G19" s="20"/>
@@ -1975,11 +1975,11 @@
       <c r="A20" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
       <c r="E20" s="19"/>
       <c r="F20" s="19"/>
       <c r="G20" s="20"/>
@@ -2067,11 +2067,11 @@
       <c r="A23" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2155,11 +2155,11 @@
       <c r="A26" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
       <c r="E26" s="12"/>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -2275,11 +2275,11 @@
       <c r="A30" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
       <c r="E30" s="23"/>
       <c r="F30" s="23"/>
       <c r="G30" s="12"/>
@@ -2307,11 +2307,11 @@
       <c r="A31" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
       <c r="E31" s="23"/>
       <c r="F31" s="23"/>
       <c r="G31" s="12"/>
@@ -5025,7 +5025,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011941A8-04BF-45E8-9F60-D4E07475AB4A}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:J46"/>
+  <dimension ref="B2:J48"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.54296875" bestFit="1" customWidth="1"/>
@@ -5101,42 +5101,34 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="I13" t="s">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H11">
+        <v>5</v>
+      </c>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H12">
+        <v>6</v>
+      </c>
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="I15" t="s">
         <v>82</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J15" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="H14">
-        <v>2018</v>
-      </c>
-      <c r="I14">
-        <v>20</v>
-      </c>
-      <c r="J14">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="H15">
-        <v>2019</v>
-      </c>
-      <c r="I15">
-        <v>20</v>
-      </c>
-      <c r="J15">
-        <v>25</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="H16">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="I16">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="J16">
         <v>25</v>
@@ -5144,358 +5136,380 @@
     </row>
     <row r="17" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H17">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="I17">
-        <v>33.5</v>
+        <v>20</v>
       </c>
       <c r="J17">
-        <f>$J$16+($J$20-$J$16)*(H17-$H$16)/($H$20-$H$16)</f>
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H18">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="I18">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="J18">
-        <f t="shared" ref="J18:J19" si="0">$J$16+($J$20-$J$16)*(H18-$H$16)/($H$20-$H$16)</f>
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H19">
+        <v>2021</v>
+      </c>
+      <c r="I19">
+        <v>33.5</v>
+      </c>
+      <c r="J19">
+        <f>$J$18+($J$22-$J$18)*(H19-$H$18)/($H$22-$H$18)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H20">
+        <v>2022</v>
+      </c>
+      <c r="I20">
+        <v>41</v>
+      </c>
+      <c r="J20">
+        <f t="shared" ref="J20:J21" si="0">$J$18+($J$22-$J$18)*(H20-$H$18)/($H$22-$H$18)</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H21">
         <v>2023</v>
       </c>
-      <c r="I19">
+      <c r="I21">
         <v>48.5</v>
       </c>
-      <c r="J19">
+      <c r="J21">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H20">
-        <v>2024</v>
-      </c>
-      <c r="I20">
-        <v>56</v>
-      </c>
-      <c r="J20">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H21">
-        <v>2025</v>
-      </c>
-      <c r="I21">
-        <v>63.5</v>
-      </c>
-      <c r="J21" s="10">
-        <f>$J$20+($J$31-$J$20)*(H21-$H$20)/($H$31-$H$20)</f>
-        <v>75.181818181818187</v>
-      </c>
-    </row>
     <row r="22" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H22">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="I22">
-        <v>71</v>
-      </c>
-      <c r="J22" s="10">
-        <f t="shared" ref="J22:J30" si="1">$J$20+($J$31-$J$20)*(H22-$H$20)/($H$31-$H$20)</f>
-        <v>85.36363636363636</v>
+        <v>56</v>
+      </c>
+      <c r="J22">
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H23">
+        <v>2025</v>
+      </c>
+      <c r="I23">
+        <v>63.5</v>
+      </c>
+      <c r="J23" s="10">
+        <f>$J$22+($J$33-$J$22)*(H23-$H$22)/($H$33-$H$22)</f>
+        <v>75.181818181818187</v>
+      </c>
+    </row>
+    <row r="24" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H24">
+        <v>2026</v>
+      </c>
+      <c r="I24">
+        <v>71</v>
+      </c>
+      <c r="J24" s="10">
+        <f t="shared" ref="J24:J32" si="1">$J$22+($J$33-$J$22)*(H24-$H$22)/($H$33-$H$22)</f>
+        <v>85.36363636363636</v>
+      </c>
+    </row>
+    <row r="25" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H25">
         <v>2027</v>
       </c>
-      <c r="I23">
+      <c r="I25">
         <v>78.5</v>
       </c>
-      <c r="J23" s="10">
+      <c r="J25" s="10">
         <f t="shared" si="1"/>
         <v>95.545454545454547</v>
       </c>
     </row>
-    <row r="24" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H24">
+    <row r="26" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H26">
         <v>2028</v>
       </c>
-      <c r="I24">
+      <c r="I26">
         <v>86</v>
       </c>
-      <c r="J24" s="10">
+      <c r="J26" s="10">
         <f t="shared" si="1"/>
         <v>105.72727272727272</v>
       </c>
     </row>
-    <row r="25" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H25">
+    <row r="27" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H27">
         <v>2029</v>
       </c>
-      <c r="I25">
+      <c r="I27">
         <v>93.5</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J27" s="10">
         <f t="shared" si="1"/>
         <v>115.90909090909091</v>
       </c>
     </row>
-    <row r="26" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H26">
+    <row r="28" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H28">
         <v>2030</v>
       </c>
-      <c r="I26">
+      <c r="I28">
         <v>100</v>
       </c>
-      <c r="J26" s="10">
+      <c r="J28" s="10">
         <f t="shared" si="1"/>
         <v>126.09090909090909</v>
       </c>
     </row>
-    <row r="27" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H27">
+    <row r="29" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H29">
         <v>2031</v>
       </c>
-      <c r="I27">
+      <c r="I29">
         <v>106.5</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J29" s="10">
         <f t="shared" si="1"/>
         <v>136.27272727272725</v>
       </c>
     </row>
-    <row r="28" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H28">
+    <row r="30" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H30">
         <v>2032</v>
       </c>
-      <c r="I28">
+      <c r="I30">
         <v>113</v>
       </c>
-      <c r="J28" s="10">
+      <c r="J30" s="10">
         <f t="shared" si="1"/>
         <v>146.45454545454544</v>
       </c>
     </row>
-    <row r="29" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H29">
+    <row r="31" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H31">
         <v>2033</v>
       </c>
-      <c r="I29">
+      <c r="I31">
         <v>119.5</v>
       </c>
-      <c r="J29" s="10">
+      <c r="J31" s="10">
         <f t="shared" si="1"/>
         <v>156.63636363636363</v>
       </c>
     </row>
-    <row r="30" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H30">
+    <row r="32" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H32">
         <v>2034</v>
       </c>
-      <c r="I30">
+      <c r="I32">
         <v>126</v>
       </c>
-      <c r="J30" s="10">
+      <c r="J32" s="10">
         <f t="shared" si="1"/>
         <v>166.81818181818181</v>
       </c>
     </row>
-    <row r="31" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H31">
-        <v>2035</v>
-      </c>
-      <c r="I31">
-        <v>132.5</v>
-      </c>
-      <c r="J31">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="32" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H32">
-        <v>2036</v>
-      </c>
-      <c r="I32">
-        <v>139</v>
-      </c>
-      <c r="J32" s="10">
-        <f>+$J$31*I32/$I$31</f>
-        <v>185.68301886792452</v>
-      </c>
-    </row>
     <row r="33" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H33">
-        <v>2037</v>
+        <v>2035</v>
       </c>
       <c r="I33">
-        <v>145.5</v>
-      </c>
-      <c r="J33" s="10">
-        <f t="shared" ref="J33:J46" si="2">+$J$31*I33/$I$31</f>
-        <v>194.36603773584906</v>
+        <v>132.5</v>
+      </c>
+      <c r="J33">
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H34">
+        <v>2036</v>
+      </c>
+      <c r="I34">
+        <v>139</v>
+      </c>
+      <c r="J34" s="10">
+        <f>+$J$33*I34/$I$33</f>
+        <v>185.68301886792452</v>
+      </c>
+    </row>
+    <row r="35" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H35">
+        <v>2037</v>
+      </c>
+      <c r="I35">
+        <v>145.5</v>
+      </c>
+      <c r="J35" s="10">
+        <f t="shared" ref="J35:J48" si="2">+$J$33*I35/$I$33</f>
+        <v>194.36603773584906</v>
+      </c>
+    </row>
+    <row r="36" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H36">
         <v>2038</v>
       </c>
-      <c r="I34">
+      <c r="I36">
         <v>152</v>
       </c>
-      <c r="J34" s="10">
+      <c r="J36" s="10">
         <f t="shared" si="2"/>
         <v>203.04905660377358</v>
       </c>
     </row>
-    <row r="35" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H35">
+    <row r="37" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H37">
         <v>2039</v>
       </c>
-      <c r="I35">
+      <c r="I37">
         <v>158.5</v>
       </c>
-      <c r="J35" s="10">
+      <c r="J37" s="10">
         <f t="shared" si="2"/>
         <v>211.73207547169812</v>
       </c>
     </row>
-    <row r="36" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H36">
+    <row r="38" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H38">
         <v>2040</v>
       </c>
-      <c r="I36">
+      <c r="I38">
         <v>166</v>
       </c>
-      <c r="J36" s="10">
+      <c r="J38" s="10">
         <f t="shared" si="2"/>
         <v>221.7509433962264</v>
       </c>
     </row>
-    <row r="37" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H37">
+    <row r="39" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H39">
         <v>2041</v>
       </c>
-      <c r="I37">
+      <c r="I39">
         <v>173.5</v>
       </c>
-      <c r="J37" s="10">
+      <c r="J39" s="10">
         <f t="shared" si="2"/>
         <v>231.76981132075471</v>
       </c>
     </row>
-    <row r="38" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H38">
+    <row r="40" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H40">
         <v>2042</v>
       </c>
-      <c r="I38">
+      <c r="I40">
         <v>181</v>
       </c>
-      <c r="J38" s="10">
+      <c r="J40" s="10">
         <f t="shared" si="2"/>
         <v>241.78867924528302</v>
       </c>
     </row>
-    <row r="39" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H39">
+    <row r="41" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H41">
         <v>2043</v>
       </c>
-      <c r="I39">
+      <c r="I41">
         <v>188.5</v>
       </c>
-      <c r="J39" s="10">
+      <c r="J41" s="10">
         <f t="shared" si="2"/>
         <v>251.80754716981133</v>
       </c>
     </row>
-    <row r="40" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H40">
+    <row r="42" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H42">
         <v>2044</v>
       </c>
-      <c r="I40">
+      <c r="I42">
         <v>196</v>
       </c>
-      <c r="J40" s="10">
+      <c r="J42" s="10">
         <f t="shared" si="2"/>
         <v>261.82641509433961</v>
       </c>
     </row>
-    <row r="41" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H41">
+    <row r="43" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H43">
         <v>2045</v>
       </c>
-      <c r="I41">
+      <c r="I43">
         <v>204.5</v>
       </c>
-      <c r="J41" s="10">
+      <c r="J43" s="10">
         <f t="shared" si="2"/>
         <v>273.18113207547168</v>
       </c>
     </row>
-    <row r="42" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H42">
+    <row r="44" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H44">
         <v>2046</v>
       </c>
-      <c r="I42">
+      <c r="I44">
         <v>214</v>
       </c>
-      <c r="J42" s="10">
+      <c r="J44" s="10">
         <f t="shared" si="2"/>
         <v>285.87169811320757</v>
       </c>
     </row>
-    <row r="43" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H43">
+    <row r="45" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H45">
         <v>2047</v>
       </c>
-      <c r="I43">
+      <c r="I45">
         <v>224.5</v>
       </c>
-      <c r="J43" s="10">
+      <c r="J45" s="10">
         <f t="shared" si="2"/>
         <v>299.89811320754717</v>
       </c>
     </row>
-    <row r="44" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H44">
+    <row r="46" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H46">
         <v>2048</v>
       </c>
-      <c r="I44">
+      <c r="I46">
         <v>236</v>
       </c>
-      <c r="J44" s="10">
+      <c r="J46" s="10">
         <f t="shared" si="2"/>
         <v>315.26037735849059</v>
       </c>
     </row>
-    <row r="45" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H45">
+    <row r="47" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H47">
         <v>2049</v>
       </c>
-      <c r="I45">
+      <c r="I47">
         <v>248.5</v>
       </c>
-      <c r="J45" s="10">
+      <c r="J47" s="10">
         <f t="shared" si="2"/>
         <v>331.95849056603771</v>
       </c>
     </row>
-    <row r="46" spans="8:10" x14ac:dyDescent="0.35">
-      <c r="H46">
+    <row r="48" spans="8:10" x14ac:dyDescent="0.35">
+      <c r="H48">
         <v>2050</v>
       </c>
-      <c r="I46">
+      <c r="I48">
         <v>262</v>
       </c>
-      <c r="J46" s="10">
+      <c r="J48" s="10">
         <f t="shared" si="2"/>
         <v>349.99245283018865</v>
       </c>
@@ -5650,136 +5664,136 @@
       <c r="F4" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="30">
-        <f>(+VLOOKUP(G3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="G4" s="27">
+        <f>(+VLOOKUP(G3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>0.02</v>
       </c>
-      <c r="H4" s="30">
-        <f>(+VLOOKUP(H3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="H4" s="27">
+        <f>(+VLOOKUP(H3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>0.02</v>
       </c>
-      <c r="I4" s="30">
-        <f>(+VLOOKUP(I3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="I4" s="27">
+        <f>(+VLOOKUP(I3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="J4" s="30">
-        <f>(+VLOOKUP(J3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="J4" s="27">
+        <f>(+VLOOKUP(J3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>3.3500000000000002E-2</v>
       </c>
-      <c r="K4" s="30">
-        <f>(+VLOOKUP(K3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="K4" s="27">
+        <f>(+VLOOKUP(K3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="L4" s="30">
-        <f>(+VLOOKUP(L3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="L4" s="27">
+        <f>(+VLOOKUP(L3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>4.8500000000000001E-2</v>
       </c>
-      <c r="M4" s="30">
-        <f>(+VLOOKUP(M3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="M4" s="27">
+        <f>(+VLOOKUP(M3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="N4" s="30">
-        <f>(+VLOOKUP(N3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="N4" s="27">
+        <f>(+VLOOKUP(N3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>6.3500000000000001E-2</v>
       </c>
-      <c r="O4" s="30">
-        <f>(+VLOOKUP(O3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="O4" s="27">
+        <f>(+VLOOKUP(O3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="P4" s="30">
-        <f>(+VLOOKUP(P3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="P4" s="27">
+        <f>(+VLOOKUP(P3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>7.85E-2</v>
       </c>
-      <c r="Q4" s="30">
-        <f>(+VLOOKUP(Q3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="Q4" s="27">
+        <f>(+VLOOKUP(Q3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="R4" s="30">
-        <f>(+VLOOKUP(R3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="R4" s="27">
+        <f>(+VLOOKUP(R3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>9.35E-2</v>
       </c>
-      <c r="S4" s="30">
-        <f>(+VLOOKUP(S3,config!$H$13:$J$46,2,FALSE))/1000</f>
+      <c r="S4" s="27">
+        <f>(+VLOOKUP(S3,config!$H$15:$J$48,2,FALSE))/1000</f>
         <v>0.1</v>
       </c>
-      <c r="T4" s="30">
-        <f>(+VLOOKUP(T3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="T4" s="27">
+        <f>(+VLOOKUP(T3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.1065</v>
       </c>
-      <c r="U4" s="30">
-        <f>(+VLOOKUP(U3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="U4" s="27">
+        <f>(+VLOOKUP(U3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.113</v>
       </c>
-      <c r="V4" s="30">
-        <f>(+VLOOKUP(V3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="V4" s="27">
+        <f>(+VLOOKUP(V3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.1195</v>
       </c>
-      <c r="W4" s="30">
-        <f>(+VLOOKUP(W3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="W4" s="27">
+        <f>(+VLOOKUP(W3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.126</v>
       </c>
-      <c r="X4" s="30">
-        <f>(+VLOOKUP(X3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="X4" s="27">
+        <f>(+VLOOKUP(X3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.13250000000000001</v>
       </c>
-      <c r="Y4" s="30">
-        <f>(+VLOOKUP(Y3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="Y4" s="27">
+        <f>(+VLOOKUP(Y3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.13900000000000001</v>
       </c>
-      <c r="Z4" s="30">
-        <f>(+VLOOKUP(Z3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="Z4" s="27">
+        <f>(+VLOOKUP(Z3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.14549999999999999</v>
       </c>
-      <c r="AA4" s="30">
-        <f>(+VLOOKUP(AA3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AA4" s="27">
+        <f>(+VLOOKUP(AA3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.152</v>
       </c>
-      <c r="AB4" s="30">
-        <f>(+VLOOKUP(AB3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AB4" s="27">
+        <f>(+VLOOKUP(AB3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.1585</v>
       </c>
-      <c r="AC4" s="30">
-        <f>(+VLOOKUP(AC3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AC4" s="27">
+        <f>(+VLOOKUP(AC3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.16600000000000001</v>
       </c>
-      <c r="AD4" s="30">
-        <f>(+VLOOKUP(AD3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AD4" s="27">
+        <f>(+VLOOKUP(AD3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.17349999999999999</v>
       </c>
-      <c r="AE4" s="30">
-        <f>(+VLOOKUP(AE3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AE4" s="27">
+        <f>(+VLOOKUP(AE3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.18099999999999999</v>
       </c>
-      <c r="AF4" s="30">
-        <f>(+VLOOKUP(AF3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AF4" s="27">
+        <f>(+VLOOKUP(AF3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.1885</v>
       </c>
-      <c r="AG4" s="30">
-        <f>(+VLOOKUP(AG3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AG4" s="27">
+        <f>(+VLOOKUP(AG3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.19600000000000001</v>
       </c>
-      <c r="AH4" s="30">
-        <f>(+VLOOKUP(AH3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AH4" s="27">
+        <f>(+VLOOKUP(AH3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.20449999999999999</v>
       </c>
-      <c r="AI4" s="30">
-        <f>(+VLOOKUP(AI3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AI4" s="27">
+        <f>(+VLOOKUP(AI3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.214</v>
       </c>
-      <c r="AJ4" s="30">
-        <f>(+VLOOKUP(AJ3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AJ4" s="27">
+        <f>(+VLOOKUP(AJ3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.22450000000000001</v>
       </c>
-      <c r="AK4" s="30">
-        <f>(+VLOOKUP(AK3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AK4" s="27">
+        <f>(+VLOOKUP(AK3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.23599999999999999</v>
       </c>
-      <c r="AL4" s="30">
-        <f>(+VLOOKUP(AL3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AL4" s="27">
+        <f>(+VLOOKUP(AL3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.2485</v>
       </c>
-      <c r="AM4" s="30">
-        <f>(+VLOOKUP(AM3,config!$H$13:$J$46,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
+      <c r="AM4" s="27">
+        <f>(+VLOOKUP(AM3,config!$H$15:$J$48,2,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,2,FALSE)))/1000</f>
         <v>0.26200000000000001</v>
       </c>
     </row>
@@ -5793,136 +5807,136 @@
       <c r="F5" t="s">
         <v>87</v>
       </c>
-      <c r="G5" s="30">
-        <f>(+VLOOKUP(G3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="G5" s="27">
+        <f>(+VLOOKUP(G3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="H5" s="30">
-        <f>(+VLOOKUP(H3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="H5" s="27">
+        <f>(+VLOOKUP(H3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="I5" s="30">
-        <f>(+VLOOKUP(I3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="I5" s="27">
+        <f>(+VLOOKUP(I3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="J5" s="30">
-        <f>(+VLOOKUP(J3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="J5" s="27">
+        <f>(+VLOOKUP(J3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="K5" s="30">
-        <f>(+VLOOKUP(K3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="K5" s="27">
+        <f>(+VLOOKUP(K3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="L5" s="30">
-        <f>(+VLOOKUP(L3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="L5" s="27">
+        <f>(+VLOOKUP(L3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>5.5E-2</v>
       </c>
-      <c r="M5" s="30">
-        <f>(+VLOOKUP(M3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="M5" s="27">
+        <f>(+VLOOKUP(M3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="N5" s="30">
-        <f>(+VLOOKUP(N3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="N5" s="27">
+        <f>(+VLOOKUP(N3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>7.5181818181818183E-2</v>
       </c>
-      <c r="O5" s="30">
-        <f>(+VLOOKUP(O3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="O5" s="27">
+        <f>(+VLOOKUP(O3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>8.5363636363636364E-2</v>
       </c>
-      <c r="P5" s="30">
-        <f>(+VLOOKUP(P3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="P5" s="27">
+        <f>(+VLOOKUP(P3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>9.5545454545454545E-2</v>
       </c>
-      <c r="Q5" s="30">
-        <f>(+VLOOKUP(Q3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="Q5" s="27">
+        <f>(+VLOOKUP(Q3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>0.10572727272727273</v>
       </c>
-      <c r="R5" s="30">
-        <f>(+VLOOKUP(R3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="R5" s="27">
+        <f>(+VLOOKUP(R3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>0.11590909090909091</v>
       </c>
-      <c r="S5" s="30">
-        <f>(+VLOOKUP(S3,config!$H$13:$J$46,3,FALSE))/1000</f>
+      <c r="S5" s="27">
+        <f>(+VLOOKUP(S3,config!$H$15:$J$48,3,FALSE))/1000</f>
         <v>0.12609090909090909</v>
       </c>
-      <c r="T5" s="30">
-        <f>(+VLOOKUP(T3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="T5" s="27">
+        <f>(+VLOOKUP(T3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.13627272727272724</v>
       </c>
-      <c r="U5" s="30">
-        <f>(+VLOOKUP(U3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="U5" s="27">
+        <f>(+VLOOKUP(U3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.14645454545454545</v>
       </c>
-      <c r="V5" s="30">
-        <f>(+VLOOKUP(V3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="V5" s="27">
+        <f>(+VLOOKUP(V3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.15663636363636363</v>
       </c>
-      <c r="W5" s="30">
-        <f>(+VLOOKUP(W3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="W5" s="27">
+        <f>(+VLOOKUP(W3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.16681818181818181</v>
       </c>
-      <c r="X5" s="30">
-        <f>(+VLOOKUP(X3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="X5" s="27">
+        <f>(+VLOOKUP(X3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.17699999999999999</v>
       </c>
-      <c r="Y5" s="30">
-        <f>(+VLOOKUP(Y3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="Y5" s="27">
+        <f>(+VLOOKUP(Y3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.18568301886792452</v>
       </c>
-      <c r="Z5" s="30">
-        <f>(+VLOOKUP(Z3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="Z5" s="27">
+        <f>(+VLOOKUP(Z3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.19436603773584907</v>
       </c>
-      <c r="AA5" s="30">
-        <f>(+VLOOKUP(AA3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AA5" s="27">
+        <f>(+VLOOKUP(AA3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.20304905660377359</v>
       </c>
-      <c r="AB5" s="30">
-        <f>(+VLOOKUP(AB3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AB5" s="27">
+        <f>(+VLOOKUP(AB3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.21173207547169812</v>
       </c>
-      <c r="AC5" s="30">
-        <f>(+VLOOKUP(AC3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AC5" s="27">
+        <f>(+VLOOKUP(AC3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.22175094339622639</v>
       </c>
-      <c r="AD5" s="30">
-        <f>(+VLOOKUP(AD3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AD5" s="27">
+        <f>(+VLOOKUP(AD3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.23176981132075472</v>
       </c>
-      <c r="AE5" s="30">
-        <f>(+VLOOKUP(AE3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AE5" s="27">
+        <f>(+VLOOKUP(AE3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.24178867924528302</v>
       </c>
-      <c r="AF5" s="30">
-        <f>(+VLOOKUP(AF3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AF5" s="27">
+        <f>(+VLOOKUP(AF3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.25180754716981135</v>
       </c>
-      <c r="AG5" s="30">
-        <f>(+VLOOKUP(AG3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AG5" s="27">
+        <f>(+VLOOKUP(AG3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.26182641509433963</v>
       </c>
-      <c r="AH5" s="30">
-        <f>(+VLOOKUP(AH3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AH5" s="27">
+        <f>(+VLOOKUP(AH3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.27318113207547168</v>
       </c>
-      <c r="AI5" s="30">
-        <f>(+VLOOKUP(AI3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AI5" s="27">
+        <f>(+VLOOKUP(AI3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.28587169811320756</v>
       </c>
-      <c r="AJ5" s="30">
-        <f>(+VLOOKUP(AJ3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AJ5" s="27">
+        <f>(+VLOOKUP(AJ3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.29989811320754717</v>
       </c>
-      <c r="AK5" s="30">
-        <f>(+VLOOKUP(AK3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AK5" s="27">
+        <f>(+VLOOKUP(AK3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.31526037735849061</v>
       </c>
-      <c r="AL5" s="30">
-        <f>(+VLOOKUP(AL3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AL5" s="27">
+        <f>(+VLOOKUP(AL3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.33195849056603771</v>
       </c>
-      <c r="AM5" s="30">
-        <f>(+VLOOKUP(AM3,config!$H$13:$J$46,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
+      <c r="AM5" s="27">
+        <f>(+VLOOKUP(AM3,config!$H$15:$J$48,3,FALSE)*(1+VLOOKUP(config!$B$3,config!$H$6:$J$10,3,FALSE)))/1000</f>
         <v>0.34999245283018865</v>
       </c>
     </row>

</xml_diff>